<commit_message>
Week 5/6: weekly report, filled Reproduction_Log.xlsx, comparison table vs paper
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -621,7 +621,11 @@
           <t>T1-001</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Tier 1 — smoke test</t>
@@ -647,8 +651,8 @@
           <t>query_executed_without_error</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="n"/>
       <c r="J6" s="6">
         <f>IF(AND(ISNUMBER(H6),ISNUMBER(I6),I6&lt;&gt;0),(H6-I6)/I6*100,"")</f>
         <v/>
@@ -657,13 +661,27 @@
         <f>IF(ISNUMBER(J6),IF(ABS(J6)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
-      <c r="M6" s="5" t="inlineStr"/>
-      <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab)</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
-          <t>Liveness check for the Week-4 gate. Modern transformers, simplified prompt — not a faithful run.</t>
+          <t>Week-4 gate liveness check: generated SQL executed on SQLite. Not a faithful run.</t>
         </is>
       </c>
     </row>
@@ -673,20 +691,24 @@
           <t>T2-001</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction</t>
+          <t>Tier 2 — reproduction (run 1/3)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Spider dev</t>
+          <t>Spider dev (1034)</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
@@ -697,8 +719,12 @@
           <t>Execution Accuracy (EX)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>77.90000000000001</v>
+      </c>
       <c r="J7" s="6">
         <f>IF(AND(ISNUMBER(H7),ISNUMBER(I7),I7&lt;&gt;0),(H7-I7)/I7*100,"")</f>
         <v/>
@@ -707,21 +733,27 @@
         <f>IF(ISNUMBER(J7),IF(ABS(J7)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="n">
+        <v>6538</v>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Apple M4 (MPS, bf16)</t>
+        </is>
+      </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>1.13.1</t>
+          <t>2.13.0</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
-          <t>4.28.1</t>
+          <t>5.15.0</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Run 1 of 3.</t>
+          <t>Prompt = schema + foreign keys only; beams=4, beam 0 kept. OUTSIDE tolerance — cause: value retriever (matched contents) missing from prompt.</t>
         </is>
       </c>
     </row>
@@ -731,32 +763,40 @@
           <t>T2-002</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction</t>
+          <t>Tier 2 — reproduction (run 2/3)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Spider dev</t>
+          <t>Spider dev (1034)</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Execution Accuracy (EX)</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>77.90000000000001</v>
+      </c>
       <c r="J8" s="6">
         <f>IF(AND(ISNUMBER(H8),ISNUMBER(I8),I8&lt;&gt;0),(H8-I8)/I8*100,"")</f>
         <v/>
@@ -765,21 +805,27 @@
         <f>IF(ISNUMBER(J8),IF(ABS(J8)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
-      <c r="M8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>1.13.1</t>
+          <t>TBD (Colab default)</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>4.28.1</t>
+          <t>TBD (Colab default)</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>Run 2 of 3.</t>
+          <t>Full CodeS prompt (schema+types+PK+representative values+matched contents+question, BOS); beams=4, beam 0 kept. 741/1034; 93.5% executable.</t>
         </is>
       </c>
     </row>
@@ -789,32 +835,40 @@
           <t>T2-003</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction</t>
+          <t>Tier 2 — reproduction (run 3/3)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Spider dev</t>
+          <t>Spider dev (1034)</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Execution Accuracy (EX)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>77.90000000000001</v>
+      </c>
       <c r="J9" s="6">
         <f>IF(AND(ISNUMBER(H9),ISNUMBER(I9),I9&lt;&gt;0),(H9-I9)/I9*100,"")</f>
         <v/>
@@ -823,21 +877,27 @@
         <f>IF(ISNUMBER(J9),IF(ABS(J9)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="n">
+        <v>2111</v>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>1.13.1</t>
+          <t>TBD (Colab default)</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>4.28.1</t>
+          <t>TBD (Colab default)</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Run 3 of 3.</t>
+          <t>Full prompt + authors' selection rule (4 beams, first passing EXPLAIN QUERY PLAN) + post_process. 763/1034; 97.3% executable. Remaining deviations: no SIC schema filter; distinct-scan instead of Lucene BM25; newer torch/transformers.</t>
         </is>
       </c>
     </row>
@@ -847,20 +907,24 @@
           <t>T2-004</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction</t>
+          <t>Tier 2 — reproduction (3B row)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b</t>
+          <t>seeklhy/codes-3b-spider</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Spider dev</t>
+          <t>Spider dev (1034)</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
@@ -868,11 +932,13 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Exact-set Match (EM)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
+          <t>Execution Accuracy (EX)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="n">
+        <v>83.40000000000001</v>
+      </c>
       <c r="J10" s="6">
         <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10),I10&lt;&gt;0),(H10-I10)/I10*100,"")</f>
         <v/>
@@ -881,19 +947,19 @@
         <f>IF(ISNUMBER(J10),IF(ABS(J10)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>1.13.1</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>4.28.1</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="n"/>
+      <c r="O10" s="5" t="n"/>
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>Planned. Same harness as T2-003.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -901,7 +967,11 @@
           <t>AB-001</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Week 7 — ablation</t>
@@ -909,12 +979,12 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Spider dev</t>
+          <t>Spider dev (1034)</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
@@ -922,11 +992,15 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Execution Accuracy (EX) — schema filter DISABLED</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr"/>
+          <t>EX — value retriever DISABLED</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>71.7</v>
+      </c>
       <c r="J11" s="6">
         <f>IF(AND(ISNUMBER(H11),ISNUMBER(I11),I11&lt;&gt;0),(H11-I11)/I11*100,"")</f>
         <v/>
@@ -935,22 +1009,98 @@
         <f>IF(ISNUMBER(J11),IF(ABS(J11)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="n">
+        <v>6538</v>
+      </c>
+      <c r="M11" s="5" t="inlineStr">
+        <is>
+          <t>Apple M4 (MPS)</t>
+        </is>
+      </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>1.13.1</t>
+          <t>2.13.0</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>4.28.1</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>Ablation: expect a measurable drop versus T2-001, confirming the module contributes.</t>
-        </is>
+          <t>5.15.0</t>
+        </is>
+      </c>
+      <c r="P11" s="7">
+        <f> T2-001 vs T2-002: removing matched contents costs 6.9 points (paper value column = our full-prompt baseline, not the paper).</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AB-002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Week 7 — ablation</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>42</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>EX — candidate selection DISABLED</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="J12">
+        <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12),I12&lt;&gt;0),(H12-I12)/I12*100,"")</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>IF(ISNUMBER(J12),IF(ABS(J12)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L12" t="n">
+        <v>2211</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="P12">
+        <f> T2-002 vs T2-003: keeping beam 0 instead of first-executable candidate costs 2.1 points (baseline = T2-003).</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1060,7 +1210,11 @@
           <t>8 × NVIDIA A800, 80GB VRAM</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr"/>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Tesla T4 16GB (Colab) for T2-002/003; Apple M4 (MPS) for T2-001</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -1073,7 +1227,11 @@
           <t>11.8</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr"/>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Colab default (TBD)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
@@ -1086,7 +1244,11 @@
           <t>Intel Xeon Platinum 8358</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr"/>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Apple M4 (local) / Colab VM (TBD)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -1099,7 +1261,11 @@
           <t>1024 GB</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr"/>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>16 GB (local)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -1112,7 +1278,11 @@
           <t>CentOS Linux 7</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr"/>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>macOS 26.6.2 (local) / Ubuntu (Colab)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -1125,7 +1295,11 @@
           <t>3.8.5 (Anaconda3)</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr"/>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>3.13.5 (local) / Colab default</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -1138,7 +1312,11 @@
           <t>1.13.1</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr"/>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>2.13.0 (local) / Colab default</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -1151,7 +1329,11 @@
           <t>4.28.1</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr"/>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>5.15.0 (local) / Colab default</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -1298,7 +1480,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done (T1-001, 2026-08-14)</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1502,7 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done (T2-001/002/003)</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1524,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>v1 drafted; update pending</t>
         </is>
       </c>
     </row>
@@ -1434,6 +1616,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Reproducibility Report v2, Excel log and ablation note updated for T2-005
- docs/Code_Reproducibility_Report_v2.docx: headline official EX 77.8% vs 77.9%,
  harness-audit section, ablation table, new deviations; v1 kept as submitted.
- Reproduction_Log.xlsx: all runs through T2-005, metric per run labelled,
  pending v2 ablations AB-103..106, env and milestones filled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>5.15.0</t>
         </is>
       </c>
       <c r="P6" s="7" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction (run 1/3)</t>
+          <t>Tier 2 — harness v1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Execution Accuracy (EX)</t>
+          <t>EX (simple metric)</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
@@ -753,7 +753,7 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Prompt = schema + foreign keys only; beams=4, beam 0 kept. OUTSIDE tolerance — cause: value retriever (matched contents) missing from prompt.</t>
+          <t>Prompt = schema + foreign keys only; beam 0. Simple sorted-rows metric — NOT the paper's evaluator (see harness_audit.md).</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction (run 2/3)</t>
+          <t>Tier 2 — harness v1</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Execution Accuracy (EX)</t>
+          <t>EX (simple metric)</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
@@ -815,17 +815,17 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>TBD (Colab default)</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
-          <t>TBD (Colab default)</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
-          <t>Full CodeS prompt (schema+types+PK+representative values+matched contents+question, BOS); beams=4, beam 0 kept. 741/1034; 93.5% executable.</t>
+          <t>Full CodeS prompt; beam 0. 741/1034; 93.5% executable. Simple metric; numeric-value retriever bug present.</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction (run 3/3)</t>
+          <t>Tier 2 — harness v1</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -860,11 +860,11 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Execution Accuracy (EX)</t>
+          <t>EX (simple metric)</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>73.8</v>
+        <v>73.79000000000001</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>77.90000000000001</v>
@@ -887,39 +887,39 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>TBD (Colab default)</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
-          <t>TBD (Colab default)</t>
+          <t>not recorded</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Full prompt + authors' selection rule (4 beams, first passing EXPLAIN QUERY PLAN) + post_process. 763/1034; 97.3% executable. Remaining deviations: no SIC schema filter; distinct-scan instead of Lucene BM25; newer torch/transformers.</t>
+          <t>+ authors' selection rule (first of 4 beams passing EXPLAIN QUERY PLAN). 763/1034; 97.3% executable. Simple metric; retriever bug present.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>T2-004</t>
+          <t>T2-003r</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — reproduction (3B row)</t>
+          <t>Tier 2 — harness v1 (repeat)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-3b-spider</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -932,12 +932,14 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Execution Accuracy (EX)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="n"/>
+          <t>EX (simple metric)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>73.79000000000001</v>
+      </c>
       <c r="I10" s="5" t="n">
-        <v>83.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J10" s="6">
         <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10),I10&lt;&gt;0),(H10-I10)/I10*100,"")</f>
@@ -947,34 +949,44 @@
         <f>IF(ISNUMBER(J10),IF(ABS(J10)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L10" s="5" t="n"/>
+      <c r="L10" s="5" t="n">
+        <v>2270</v>
+      </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
-          <t>Planned. Same harness as T2-003.</t>
+          <t>Identical repeat of T2-003: 763/1034 again — decoding is deterministic.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>AB-001</t>
+          <t>T2-005</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Week 7 — ablation</t>
+          <t>Tier 2 — harness v2 (HEADLINE)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -992,14 +1004,14 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>EX — value retriever DISABLED</t>
+          <t>EX (OFFICIAL Spider evaluator)</t>
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>64.8</v>
+        <v>77.8</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>71.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J11" s="6">
         <f>IF(AND(ISNUMBER(H11),ISNUMBER(I11),I11&lt;&gt;0),(H11-I11)/I11*100,"")</f>
@@ -1010,144 +1022,662 @@
         <v/>
       </c>
       <c r="L11" s="5" t="n">
-        <v>6538</v>
+        <v>2865</v>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Apple M4 (MPS)</t>
+          <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>2.13.0</t>
+          <t>2.11.0+cu128</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>5.15.0</t>
-        </is>
-      </c>
-      <c r="P11" s="7">
-        <f> T2-001 vs T2-002: removing matched contents costs 6.9 points (paper value column = our full-prompt baseline, not the paper).</f>
-        <v/>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>After audit: numeric values in retriever, tables.json comments, authors' truncation; scored with test_suite_sql_eval evaluation.py --etype exec (paper's metric). Simple metric on same preds = 73.4. 97.3% executable.</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>AB-002</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Week 7 — ablation</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>T2-004</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Tier 2 — 3B row (planned)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-3b-spider</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>EX (OFFICIAL)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="J12" s="6">
+        <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12),I12&lt;&gt;0),(H12-I12)/I12*100,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>IF(ISNUMBER(J12),IF(ABS(J12)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="5" t="n"/>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
+          <t>Planned, harness v2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>AB-003</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v1</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Spider dev (1034)</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="F13" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>EX — candidate selection DISABLED</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>71.7</v>
-      </c>
-      <c r="I12" t="n">
-        <v>73.8</v>
-      </c>
-      <c r="J12">
-        <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12),I12&lt;&gt;0),(H12-I12)/I12*100,"")</f>
-        <v/>
-      </c>
-      <c r="K12">
-        <f>IF(ISNUMBER(J12),IF(ABS(J12)&lt;=10,"YES","NO — document cause"),"")</f>
-        <v/>
-      </c>
-      <c r="L12" t="n">
-        <v>2211</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Tesla T4 (Colab)</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>EX simple — no representative values</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>72.23999999999999</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="J13" s="6">
+        <f>IF(AND(ISNUMBER(H13),ISNUMBER(I13),I13&lt;&gt;0),(H13-I13)/I13*100,"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>IF(ISNUMBER(J13),IF(ABS(J13)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>1652</v>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>Paper Value column = our baseline T2-003 (not the paper). 747/1034; 97.8% executable. Δ −1.55.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>AB-004</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v1</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>EX simple — no matched contents</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>71.08</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="J14" s="6">
+        <f>IF(AND(ISNUMBER(H14),ISNUMBER(I14),I14&lt;&gt;0),(H14-I14)/I14*100,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>IF(ISNUMBER(J14),IF(ABS(J14)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>2234</v>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P14" s="7" t="inlineStr">
+        <is>
+          <t>Baseline T2-003. 735/1034; 96.8% executable. Δ −2.71 (largest).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>AB-005</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v1</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>EX simple — no foreign keys</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>72.23999999999999</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="J15" s="6">
+        <f>IF(AND(ISNUMBER(H15),ISNUMBER(I15),I15&lt;&gt;0),(H15-I15)/I15*100,"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>IF(ISNUMBER(J15),IF(ABS(J15)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>2062</v>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>Baseline T2-003. 747/1034; 95.5% executable. Δ −1.55.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>AB-006</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v1</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>EX simple — no candidate selection</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>71.66</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="J16" s="6">
+        <f>IF(AND(ISNUMBER(H16),ISNUMBER(I16),I16&lt;&gt;0),(H16-I16)/I16*100,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="5">
+        <f>IF(ISNUMBER(J16),IF(ABS(J16)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>2265</v>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t>Baseline T2-003. 741/1034 — identical to T2-002. 93.5% executable. Δ −2.13.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>AB-103</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v2</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>EX OFFICIAL — no representative values</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J17" s="6">
+        <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17),I17&lt;&gt;0),(H17-I17)/I17*100,"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>IF(ISNUMBER(J17),IF(ABS(J17)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5" t="n"/>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>AB-104</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="P12">
-        <f> T2-002 vs T2-003: keeping beam 0 instead of first-executable candidate costs 2.1 points (baseline = T2-003).</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Mean of the three Tier-2 EX runs:</t>
-        </is>
-      </c>
-      <c r="H13" s="9">
-        <f>IFERROR(AVERAGE(H7:H9),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Standard deviation:</t>
-        </is>
-      </c>
-      <c r="H14" s="9">
-        <f>IFERROR(STDEV(H7:H9),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v2</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>EX OFFICIAL — no matched contents</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J18" s="6">
+        <f>IF(AND(ISNUMBER(H18),ISNUMBER(I18),I18&lt;&gt;0),(H18-I18)/I18*100,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>IF(ISNUMBER(J18),IF(ABS(J18)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="5" t="n"/>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="n"/>
+      <c r="O18" s="5" t="n"/>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>AB-105</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v2</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>EX OFFICIAL — no foreign keys</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J19" s="6">
+        <f>IF(AND(ISNUMBER(H19),ISNUMBER(I19),I19&lt;&gt;0),(H19-I19)/I19*100,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="5">
+        <f>IF(ISNUMBER(J19),IF(ABS(J19)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="5" t="n"/>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="n"/>
+      <c r="O19" s="5" t="n"/>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>AB-106</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v2</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>EX OFFICIAL — no candidate selection</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J20" s="6">
+        <f>IF(AND(ISNUMBER(H20),ISNUMBER(I20),I20&lt;&gt;0),(H20-I20)/I20*100,"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="5">
+        <f>IF(ISNUMBER(J20),IF(ABS(J20)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="5" t="n"/>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="n"/>
+      <c r="O20" s="5" t="n"/>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
+        </is>
+      </c>
+      <c r="H21" s="9">
+        <f>H10-H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Headline vs paper (T2-005, official metric), points:</t>
+        </is>
+      </c>
+      <c r="H22" s="9">
+        <f>H11-I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>
@@ -1212,7 +1742,7 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Tesla T4 16GB (Colab) for T2-002/003; Apple M4 (MPS) for T2-001</t>
+          <t>Tesla T4 16GB (Colab) for T2-002 onward; Apple M4 (MPS) for T2-001</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1759,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Colab default (TBD)</t>
+          <t>12.8 (torch 2.11.0+cu128)</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1844,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>2.13.0 (local) / Colab default</t>
+          <t>2.11.0+cu128 (Colab, from T2-003r) / 2.13.0 (local)</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1861,7 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>5.15.0 (local) / Colab default</t>
+          <t>5.16.1 (Colab, from T2-003r) / 5.15.0 (local)</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1889,11 @@
           <t>0.21.0 (requires Java 11)</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr"/>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>not used (distinct-value scan instead)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -1387,7 +1921,7 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>CodeS-1B</t>
+          <t>CodeS-1B (SFT, Spider)</t>
         </is>
       </c>
     </row>
@@ -1480,7 +2014,7 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Done (T1-001, 2026-08-14)</t>
+          <t>Done (T1-001, 14 Aug)</t>
         </is>
       </c>
     </row>
@@ -1502,7 +2036,7 @@
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>Done (T2-001/002/003)</t>
+          <t>Done (T2-001..T2-005)</t>
         </is>
       </c>
     </row>
@@ -1524,7 +2058,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>v1 drafted; update pending</t>
+          <t>v2 written (26 Sep)</t>
         </is>
       </c>
     </row>
@@ -1616,7 +2150,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Week 7 ablations on harness v2 (official metric): -0.9 to -1.9 pts vs 77.8
AB-103 no values 76.4 | AB-104 no retriever 75.9 | AB-105 no FK 76.9 |
AB-106 no selection 76.0. Report v2, Excel/CSV log, ablation write-up updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1427,7 +1427,9 @@
           <t>EX OFFICIAL — no representative values</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n"/>
+      <c r="H17" s="5" t="n">
+        <v>76.40000000000001</v>
+      </c>
       <c r="I17" s="5" t="n">
         <v>77.8</v>
       </c>
@@ -1439,17 +1441,29 @@
         <f>IF(ISNUMBER(J17),IF(ABS(J17)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L17" s="5" t="n"/>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N17" s="5" t="n"/>
-      <c r="O17" s="5" t="n"/>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.4 pts. Simple EX 72.24 (747/1034); 98.1% executable.</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1475,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1487,7 +1501,9 @@
           <t>EX OFFICIAL — no matched contents</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n"/>
+      <c r="H18" s="5" t="n">
+        <v>75.90000000000001</v>
+      </c>
       <c r="I18" s="5" t="n">
         <v>77.8</v>
       </c>
@@ -1499,17 +1515,29 @@
         <f>IF(ISNUMBER(J18),IF(ABS(J18)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L18" s="5" t="n"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N18" s="5" t="n"/>
-      <c r="O18" s="5" t="n"/>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.9 pts. Simple EX 71.57 (740/1034); 97.2% executable.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1549,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1547,7 +1575,9 @@
           <t>EX OFFICIAL — no foreign keys</t>
         </is>
       </c>
-      <c r="H19" s="5" t="n"/>
+      <c r="H19" s="5" t="n">
+        <v>76.90000000000001</v>
+      </c>
       <c r="I19" s="5" t="n">
         <v>77.8</v>
       </c>
@@ -1559,17 +1589,29 @@
         <f>IF(ISNUMBER(J19),IF(ABS(J19)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L19" s="5" t="n"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N19" s="5" t="n"/>
-      <c r="O19" s="5" t="n"/>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -0.9 pts. Simple EX 72.34 (748/1034); 95.9% executable.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1623,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1607,7 +1649,9 @@
           <t>EX OFFICIAL — no candidate selection</t>
         </is>
       </c>
-      <c r="H20" s="5" t="n"/>
+      <c r="H20" s="5" t="n">
+        <v>76</v>
+      </c>
       <c r="I20" s="5" t="n">
         <v>77.8</v>
       </c>
@@ -1619,17 +1663,29 @@
         <f>IF(ISNUMBER(J20),IF(ABS(J20)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L20" s="5" t="n"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N20" s="5" t="n"/>
-      <c r="O20" s="5" t="n"/>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>Pending (Colab). Baseline T2-005 official 77.8.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.8 pts. Simple EX 71.66 (741/1034); 94.1% executable.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Weeks 10-11: fresh baseline T2-006 (77.76%) and abstention results
Execution-agreement abstention: 83.25% accuracy at 90.5% coverage vs 77.79%
random abstention (+5.46 pts over 10 splits; t-test p=7.7e-10, Wilcoxon
p=9.8e-4; question-level bootstrap +5.68 [+4.51,+6.71]). Beam probability
has lower AURC overall (curves cross at ~74% coverage) — reported.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1048,22 +1048,22 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>T2-004</t>
+          <t>T2-006</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — 3B row (planned)</t>
+          <t>Week 10 — fresh baseline (harness v2)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-3b-spider</t>
+          <t>seeklhy/codes-1b-spider</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1076,12 +1076,14 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>EX (OFFICIAL)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="n"/>
+          <t>EX (OFFICIAL Spider evaluator)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>77.76000000000001</v>
+      </c>
       <c r="I12" s="5" t="n">
-        <v>83.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="J12" s="6">
         <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12),I12&lt;&gt;0),(H12-I12)/I12*100,"")</f>
@@ -1091,39 +1093,51 @@
         <f>IF(ISNUMBER(J12),IF(ABS(J12)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L12" s="5" t="n"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>Planned, harness v2.</t>
+          <t>Fresh re-run of T2-005: 804/1034 official (identical); simple 759/1034 identical. Baseline for the Month-3 enhancement; candidate dump saved.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>AB-003</t>
+          <t>T2-004</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Week 7 ablation — harness v1</t>
+          <t>Tier 2 — 3B row (planned)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>seeklhy/codes-1b-spider</t>
+          <t>seeklhy/codes-3b-spider</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1136,14 +1150,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>EX simple — no representative values</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>72.23999999999999</v>
-      </c>
+          <t>EX (OFFICIAL)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n">
-        <v>73.79000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="J13" s="6">
         <f>IF(AND(ISNUMBER(H13),ISNUMBER(I13),I13&lt;&gt;0),(H13-I13)/I13*100,"")</f>
@@ -1153,34 +1165,24 @@
         <f>IF(ISNUMBER(J13),IF(ABS(J13)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L13" s="5" t="n">
-        <v>1652</v>
-      </c>
+      <c r="L13" s="5" t="n"/>
       <c r="M13" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>2.11.0+cu128</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="inlineStr">
-        <is>
-          <t>5.16.1</t>
-        </is>
-      </c>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13" s="5" t="n"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Paper Value column = our baseline T2-003 (not the paper). 747/1034; 97.8% executable. Δ −1.55.</t>
+          <t>Planned, harness v2.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>AB-004</t>
+          <t>AB-003</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1208,11 +1210,11 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>EX simple — no matched contents</t>
+          <t>EX simple — no representative values</t>
         </is>
       </c>
       <c r="H14" s="5" t="n">
-        <v>71.08</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>73.79000000000001</v>
@@ -1226,7 +1228,7 @@
         <v/>
       </c>
       <c r="L14" s="5" t="n">
-        <v>2234</v>
+        <v>1652</v>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
@@ -1245,19 +1247,19 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>Baseline T2-003. 735/1034; 96.8% executable. Δ −2.71 (largest).</t>
+          <t>Paper Value column = our baseline T2-003 (not the paper). 747/1034; 97.8% executable. Δ −1.55.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>AB-005</t>
+          <t>AB-004</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1280,11 +1282,11 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>EX simple — no foreign keys</t>
+          <t>EX simple — no matched contents</t>
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>72.23999999999999</v>
+        <v>71.08</v>
       </c>
       <c r="I15" s="5" t="n">
         <v>73.79000000000001</v>
@@ -1298,7 +1300,7 @@
         <v/>
       </c>
       <c r="L15" s="5" t="n">
-        <v>2062</v>
+        <v>2234</v>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
@@ -1317,14 +1319,14 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Baseline T2-003. 747/1034; 95.5% executable. Δ −1.55.</t>
+          <t>Baseline T2-003. 735/1034; 96.8% executable. Δ −2.71 (largest).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>AB-006</t>
+          <t>AB-005</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1352,11 +1354,11 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>EX simple — no candidate selection</t>
+          <t>EX simple — no foreign keys</t>
         </is>
       </c>
       <c r="H16" s="5" t="n">
-        <v>71.66</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>73.79000000000001</v>
@@ -1370,7 +1372,7 @@
         <v/>
       </c>
       <c r="L16" s="5" t="n">
-        <v>2265</v>
+        <v>2062</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
@@ -1389,24 +1391,24 @@
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>Baseline T2-003. 741/1034 — identical to T2-002. 93.5% executable. Δ −2.13.</t>
+          <t>Baseline T2-003. 747/1034; 95.5% executable. Δ −1.55.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>AB-103</t>
+          <t>AB-006</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Week 7 ablation — harness v2</t>
+          <t>Week 7 ablation — harness v1</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1424,14 +1426,14 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>EX OFFICIAL — no representative values</t>
+          <t>EX simple — no candidate selection</t>
         </is>
       </c>
       <c r="H17" s="5" t="n">
-        <v>76.40000000000001</v>
+        <v>71.66</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>77.8</v>
+        <v>73.79000000000001</v>
       </c>
       <c r="J17" s="6">
         <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17),I17&lt;&gt;0),(H17-I17)/I17*100,"")</f>
@@ -1441,10 +1443,8 @@
         <f>IF(ISNUMBER(J17),IF(ABS(J17)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>not reported</t>
-        </is>
+      <c r="L17" s="5" t="n">
+        <v>2265</v>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
@@ -1463,14 +1463,14 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.4 pts. Simple EX 72.24 (747/1034); 98.1% executable.</t>
+          <t>Baseline T2-003. 741/1034 — identical to T2-002. 93.5% executable. Δ −2.13.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>AB-104</t>
+          <t>AB-103</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1498,11 +1498,11 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>EX OFFICIAL — no matched contents</t>
+          <t>EX OFFICIAL — no representative values</t>
         </is>
       </c>
       <c r="H18" s="5" t="n">
-        <v>75.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>77.8</v>
@@ -1537,14 +1537,14 @@
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.9 pts. Simple EX 71.57 (740/1034); 97.2% executable.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.4 pts. Simple EX 72.24 (747/1034); 98.1% executable.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>AB-105</t>
+          <t>AB-104</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1572,11 +1572,11 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>EX OFFICIAL — no foreign keys</t>
+          <t>EX OFFICIAL — no matched contents</t>
         </is>
       </c>
       <c r="H19" s="5" t="n">
-        <v>76.90000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="I19" s="5" t="n">
         <v>77.8</v>
@@ -1611,14 +1611,14 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -0.9 pts. Simple EX 72.34 (748/1034); 95.9% executable.</t>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.9 pts. Simple EX 71.57 (740/1034); 97.2% executable.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>AB-106</t>
+          <t>AB-105</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1646,11 +1646,11 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>EX OFFICIAL — no candidate selection</t>
+          <t>EX OFFICIAL — no foreign keys</t>
         </is>
       </c>
       <c r="H20" s="5" t="n">
-        <v>76</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="I20" s="5" t="n">
         <v>77.8</v>
@@ -1685,55 +1685,130 @@
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
+          <t>Paper Value column = baseline T2-005 (77.8, official). Δ -0.9 pts. Simple EX 72.34 (748/1034); 95.9% executable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>AB-106</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Week 7 ablation — harness v2</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>EX OFFICIAL — no candidate selection</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J21" s="6">
+        <f>IF(AND(ISNUMBER(H21),ISNUMBER(I21),I21&lt;&gt;0),(H21-I21)/I21*100,"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="5">
+        <f>IF(ISNUMBER(J21),IF(ABS(J21)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>not reported</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>5.16.1</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
           <t>Paper Value column = baseline T2-005 (77.8, official). Δ -1.8 pts. Simple EX 71.66 (741/1034); 94.1% executable.</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
-        </is>
-      </c>
-      <c r="H21" s="9">
-        <f>H10-H9</f>
-        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
+        </is>
+      </c>
+      <c r="H22" s="9">
+        <f>H10-H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
           <t>Headline vs paper (T2-005, official metric), points:</t>
         </is>
       </c>
-      <c r="H22" s="9">
+      <c r="H23" s="9">
         <f>H11-I11</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>

</xml_diff>

<commit_message>
Benchmark-to-reality: Spider-Realistic run RL-001 (69.5% vs paper 70.9%)
Same 508 questions in original vs realistic wording on the same machine: 72.8% -> 69.5%, gap 3.3 pts
(bootstrap 95% CI [0.8, 5.9], exact McNemar p = 0.016); against the paper's SFT CodeS-1B Spider-
Realistic EX (Table 7) the difference is -1.4 pts. Abstention on the realistic wording: 86.2% answered,
76.7% correct, wrong answers 155 -> 102. Cross-check with T2-006 on the original twins: same SQL on
485/508, 72.8% vs 73.2%. Logged in the CSV and Excel run logs; added to the report, deck and poster.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1838,51 +1838,193 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>RL-001 (orig)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Benchmark-to-reality — Spider-Realistic twins, original wording</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev, 508 questions with a Spider-Realistic twin</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>EX (official exec match)</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="6">
+        <f>IF(AND(ISNUMBER(H23),ISNUMBER(I23),I23&lt;&gt;0),(H23-I23)/I23*100,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="5">
+        <f>IF(ISNUMBER(J23),IF(ABS(J23)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>11637</v>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Apple M4 (mps, bf16)</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>2.13.0</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>5.15.0</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>370/508. No paper value for this subset. Cross-check vs T2-006 (T4, fp16) on the same 508: same selected SQL on 485, T2-006 = 73.2 (372). Runtime covers both wordings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>RL-001 (realistic)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Benchmark-to-reality — Spider-Realistic (reproduction point)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Spider-Realistic (508), HF aherntech/spider-realistic</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>EX (official exec match)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="J24" s="6">
+        <f>IF(AND(ISNUMBER(H24),ISNUMBER(I24),I24&lt;&gt;0),(H24-I24)/I24*100,"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="5">
+        <f>IF(ISNUMBER(J24),IF(ABS(J24)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>11637</v>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>Apple M4 (mps, bf16)</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>2.13.0</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>5.15.0</t>
+        </is>
+      </c>
+      <c r="P24" s="7" t="inlineStr">
+        <is>
+          <t>353/508. Paper value: SFT CodeS-1B, Table 7 of the CodeS paper. Gap vs original wording −3.3 pts (95% CI [0.8, 5.9]), McNemar p = 0.016. Balanced abstention: 86.2% answered, 76.7% correct. results/reality/spider_realistic_RL-001.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
         </is>
       </c>
-      <c r="H23" s="9">
+      <c r="H25" s="9">
         <f>H10-H9</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Headline vs paper (T2-005, official metric), points:</t>
         </is>
       </c>
-      <c r="H24" s="9">
+      <c r="H26" s="9">
         <f>H11-I11</f>
         <v/>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>

</xml_diff>

<commit_message>
Team number is now 18 (renumbered from 21)
Updated the README, NOTICE, PRODUCT.md, CLAUDE.md, notebooks, run-log header, speaker script; added
"Team 18" to the deck's title slide and the poster's team details. Documents submitted before the
change (e.g. Week 1/Team_21.pptx, the reproducibility reports) are left as they were; the app's
internal bundle identifier is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -522,7 +522,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Team 21 · Anchor paper: CodeS (SIGMOD 2024, arXiv:2402.16347) · Benchmark: Spider dev (Hugging Face)</t>
+          <t>Team 18 · Anchor paper: CodeS (SIGMOD 2024, arXiv:2402.16347) · Benchmark: Spider dev (Hugging Face)</t>
         </is>
       </c>
     </row>
@@ -533,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -2063,6 +2064,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr"/>
       <c r="B4" s="12" t="inlineStr">
@@ -2299,6 +2301,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -2497,6 +2500,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
T2-004: CodeS-3B on Spider dev, 81.8% official EX (paper 83.4%); abstention generalises
846/1034 with the official execution match (-1.6 pts, within tolerance). Agreement abstention:
85.2% correct at 89.7% coverage (+3.2 pts, p=2.9e-6); v2 (different queries counted once):
+3.95 pts, p=1e-7, ahead of beam probability (+3.4). Logged as T2-004 and AN-002.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -1128,12 +1128,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Tier 2 — 3B row (planned)</t>
+          <t>Tier 2 — CodeS-3B (Review-III follow-up)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1151,10 +1151,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>EX (OFFICIAL)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="n"/>
+          <t>EX (OFFICIAL Spider evaluator)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>81.81999999999999</v>
+      </c>
       <c r="I13" s="5" t="n">
         <v>83.40000000000001</v>
       </c>
@@ -1166,17 +1168,29 @@
         <f>IF(ISNUMBER(J13),IF(ABS(J13)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L13" s="5" t="n"/>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
           <t>Tesla T4 (Colab, fp16)</t>
         </is>
       </c>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="5" t="n"/>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Planned, harness v2.</t>
+          <t>846/1034. Paper: Table 5, SFT CodeS-3B. Abstention: 85.2% correct at 89.7% coverage (+3.2 pts, p=2.9e-6); v2 (different queries only) +3.95 pts. results/abstention_T2-004.json, results/agreement_v2_T2-004.md</t>
         </is>
       </c>
     </row>
@@ -2002,7 +2016,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
@@ -2064,7 +2077,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="12" t="inlineStr"/>
       <c r="B4" s="12" t="inlineStr">
@@ -2301,7 +2313,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -2500,7 +2511,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
T2-004 runtime 5543 s and the official evaluation.py figure (0.8180) from the Colab output
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -1168,10 +1168,8 @@
         <f>IF(ISNUMBER(J13),IF(ABS(J13)&lt;=10,"YES","NO — document cause"),"")</f>
         <v/>
       </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>not recorded</t>
-        </is>
+      <c r="L13" s="5" t="n">
+        <v>5543</v>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Excel run log: CN-008 (failed) row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1993,50 +1993,123 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
-        </is>
-      </c>
-      <c r="H25" s="9">
-        <f>H10-H9</f>
-        <v/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>CN-008 (failed)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Review-III follow-up — CodeS-1B, 8 beams</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>EX (OFFICIAL evaluation.py)</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="6">
+        <f>IF(AND(ISNUMBER(H25),ISNUMBER(I25),I25&lt;&gt;0),(H25-I25)/I25*100,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="5">
+        <f>IF(ISNUMBER(J25),IF(ABS(J25)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>not recorded</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
+        <is>
+          <t>Generation complete; runtime died while scoring candidates, dump lost. Official 0.788 read from output (4 beams, T2-006: 0.778). Harness now saves the raw dump first. Re-run planned.</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
+        </is>
+      </c>
+      <c r="H26" s="9">
+        <f>H10-H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
           <t>Headline vs paper (T2-005, official metric), points:</t>
         </is>
       </c>
-      <c r="H26" s="9">
+      <c r="H27" s="9">
         <f>H11-I11</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>

</xml_diff>

<commit_message>
Log SM-008 attempt 1 as aborted (Colab disconnected 9 min in; no results)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2065,51 +2065,115 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
-        </is>
-      </c>
-      <c r="H26" s="9">
-        <f>H10-H9</f>
-        <v/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>SM-008 attempt 1 (aborted)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Review-III follow-up — 8 sampled candidates, T=0.8</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>none (aborted)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="n"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>~540</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t>Aborted ~9 min after start (Colab runtime disconnected at 1:51 AM; nothing saved, no metric). Probable cause: the Mac was on battery power / went to sleep overnight (battery found at 2%), which dropped the browser connection - not confirmed. Re-started 2026-10-14 20:02 on AC power.</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
+          <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
+        </is>
+      </c>
+      <c r="H27" s="9">
+        <f>H10-H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
           <t>Headline vs paper (T2-005, official metric), points:</t>
         </is>
       </c>
-      <c r="H27" s="9">
+      <c r="H28" s="9">
         <f>H11-I11</f>
         <v/>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>

</xml_diff>

<commit_message>
SM-008: CodeS-1B with 8 sampled candidates (T=0.8); abstention holds, majority vote now helps
Plain EX 77.08% (4 beams 77.76%); majority of the 8 77.66%; a correct query among the 8 for 881 questions
(4 beams: 859). Agreement abstention +5.57 pts vs random (p=1.7e-7); all 8 agree -> 93.5% correct.
For sampled candidates repeats are signal, so the dedupe-count variant is not meaningful there.
Logged as SM-008 and AN-003; tracker updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Reproduction_Log.xlsx
+++ b/results/Reproduction_Log.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2129,51 +2129,195 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>SM-008</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Review-III follow-up — 8 sampled candidates, T=0.8</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>EX (OFFICIAL exec match)</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>77.08</v>
+      </c>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="6">
+        <f>IF(AND(ISNUMBER(H27),ISNUMBER(I27),I27&lt;&gt;0),(H27-I27)/I27*100,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="5">
+        <f>IF(ISNUMBER(J27),IF(ABS(J27)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>~4400</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Tesla T4 (Colab, fp16)</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>Colab default</t>
+        </is>
+      </c>
+      <c r="P27" s="7" t="inlineStr">
+        <is>
+          <t>797/1034 (4 beams: 77.76). Majority of 8: 77.66; correct among 8: 881 (85.2%). Abstention: 82.5% correct at 90.0% coverage, +5.57 pts vs random, p=1.7e-7; all 8 agree → 93.5% correct. results/abstention_SM-008.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>AN-003</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Analysis of SM-008 — agreement v2</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>seeklhy/codes-1b-spider</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Spider dev (1034)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>selective acc (v2 share)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="6">
+        <f>IF(AND(ISNUMBER(H28),ISNUMBER(I28),I28&lt;&gt;0),(H28-I28)/I28*100,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="5">
+        <f>IF(ISNUMBER(J28),IF(ABS(J28)&lt;=10,"YES","NO — document cause"),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>Apple M4 (CPU)</t>
+        </is>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>2.13.0</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>5.15.0</t>
+        </is>
+      </c>
+      <c r="P28" s="7" t="inlineStr">
+        <is>
+          <t>v2 share +6.19 pts (p=1.5e-8) vs v1 +5.57. For sampled candidates repeats are signal; the dedupe 'count' variant is not meaningful. results/agreement_v2_SM-008.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Repeatability (T2-003 vs T2-003r, identical config):</t>
         </is>
       </c>
-      <c r="H27" s="9">
+      <c r="H29" s="9">
         <f>H10-H9</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Headline vs paper (T2-005, official metric), points:</t>
         </is>
       </c>
-      <c r="H28" s="9">
+      <c r="H30" s="9">
         <f>H11-I11</f>
         <v/>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Reminder — "reproduction complete" means:</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>• Metrics land within ±5–10% of the published values (ML/AI tolerance per the SOP), OR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>• The deviation is documented with a stated cause (different GPU, precision, library versions, batch size, dataset split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>• Read the paper value for YOUR exact configuration out of the CodeS paper — do not rely on memory or a secondary source.</t>
         </is>

</xml_diff>